<commit_message>
chore: remove Streamlit pages, refresh design mockups, update docs + weekly tracker
- Remove all 6 Streamlit pages (pages/) and .streamlit/config.toml — migrating to React + FastAPI
- Remove old flat HTML mockups (0001–0006); replace with open-design spec (.txt) and Claude-generated HTML mockup folders
- Add new design specs: orgcode-costcenter, edit-document-number pages
- Update reference docs: requirement_detail, cost center master, cost type cal, GL master, employee CSV, orgcode-CC mapping
- Remove skill/skill_design_mod1_act_bgt.md (superseded)
- Weekly tracker: mark SAP gap columns, orgcode-CC mapping, Bronze→Silver consistency check as Done; add 0003-gl-group, silver_sap_m_gl_account, gold_sap_m_gl_account_group_name entries
- Add docs/*RATIMA*.xlsx to .gitignore (140MB SAP test file exceeds GitHub limit)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/02cost center & department (master).xlsx
+++ b/docs/02cost center & department (master).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\FIN-Mgt\Budget_CMAN\Data warehouse\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\04.budget_management_web\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{387529AC-799B-4EB5-AE96-3E1B227F919C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A030B0-4238-4C40-969D-60206710639B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{5A044EB7-EC4B-476F-9C5E-70DCF7ABA329}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5A044EB7-EC4B-476F-9C5E-70DCF7ABA329}"/>
   </bookViews>
   <sheets>
     <sheet name="Cost center (Update 18 Mar 26)" sheetId="1" r:id="rId1"/>
@@ -14369,9 +14369,6 @@
     <t>10QC011000</t>
   </si>
   <si>
-    <t>Quality Control (TK&amp;KK)</t>
-  </si>
-  <si>
     <t>Production (KK)</t>
   </si>
   <si>
@@ -15447,6 +15444,9 @@
   </si>
   <si>
     <t>IBC</t>
+  </si>
+  <si>
+    <t>Raw Material and Fuel</t>
   </si>
 </sst>
 </file>
@@ -15480,12 +15480,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -15501,7 +15513,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -15511,12 +15523,38 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{41FDB980-3965-49F7-BE83-36518BCA17F1}"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -15551,9 +15589,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -15591,7 +15629,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -15697,7 +15735,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -15839,7 +15877,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -15863,19 +15901,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
@@ -16428,7 +16466,7 @@
         <v>84</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>85</v>
+        <v>257</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>70</v>
@@ -16442,10 +16480,10 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>70</v>
@@ -16454,15 +16492,15 @@
         <v>74</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>70</v>
@@ -16476,10 +16514,10 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>70</v>
@@ -16488,15 +16526,15 @@
         <v>74</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>70</v>
@@ -16505,15 +16543,15 @@
         <v>74</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>96</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>70</v>
@@ -16527,10 +16565,10 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>97</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>98</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>70</v>
@@ -16544,10 +16582,10 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>99</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>100</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>70</v>
@@ -16561,10 +16599,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>70</v>
@@ -16578,10 +16616,10 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>70</v>
@@ -16595,10 +16633,10 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>106</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>70</v>
@@ -16612,10 +16650,10 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B45" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>108</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>70</v>
@@ -16629,10 +16667,10 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>110</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>70</v>
@@ -16646,10 +16684,10 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B47" s="2" t="s">
         <v>111</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>112</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>70</v>
@@ -16663,10 +16701,10 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B48" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="B48" s="2" t="s">
-        <v>114</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>70</v>
@@ -16680,10 +16718,10 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B49" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>70</v>
@@ -16697,10 +16735,10 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B50" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>118</v>
       </c>
       <c r="C50" s="2" t="s">
         <v>70</v>
@@ -16714,10 +16752,10 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B51" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="B51" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>70</v>
@@ -16726,15 +16764,15 @@
         <v>74</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B52" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="B52" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>70</v>
@@ -16743,15 +16781,15 @@
         <v>74</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B53" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="B53" s="2" t="s">
-        <v>124</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>70</v>
@@ -16765,10 +16803,10 @@
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>126</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>70</v>
@@ -16782,10 +16820,10 @@
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>70</v>
@@ -16799,10 +16837,10 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>130</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>70</v>
@@ -16816,10 +16854,10 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B57" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="B57" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="C57" s="2" t="s">
         <v>70</v>
@@ -16833,10 +16871,10 @@
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B58" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="B58" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="C58" s="2" t="s">
         <v>70</v>
@@ -16850,10 +16888,10 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B59" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="B59" s="2" t="s">
-        <v>136</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>70</v>
@@ -16862,15 +16900,15 @@
         <v>74</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B60" s="2" t="s">
         <v>137</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>138</v>
       </c>
       <c r="C60" s="2" t="s">
         <v>70</v>
@@ -16879,15 +16917,15 @@
         <v>74</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B61" s="2" t="s">
         <v>139</v>
-      </c>
-      <c r="B61" s="2" t="s">
-        <v>140</v>
       </c>
       <c r="C61" s="2" t="s">
         <v>70</v>
@@ -16896,15 +16934,15 @@
         <v>74</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B62" s="2" t="s">
         <v>141</v>
-      </c>
-      <c r="B62" s="2" t="s">
-        <v>142</v>
       </c>
       <c r="C62" s="2" t="s">
         <v>70</v>
@@ -16913,15 +16951,15 @@
         <v>74</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B63" s="2" t="s">
         <v>143</v>
-      </c>
-      <c r="B63" s="2" t="s">
-        <v>144</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>70</v>
@@ -16930,15 +16968,15 @@
         <v>74</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B64" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="B64" s="2" t="s">
-        <v>146</v>
       </c>
       <c r="C64" s="2" t="s">
         <v>70</v>
@@ -16947,15 +16985,15 @@
         <v>74</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B65" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="B65" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>70</v>
@@ -16964,15 +17002,15 @@
         <v>74</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>149</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>150</v>
       </c>
       <c r="C66" s="2" t="s">
         <v>70</v>
@@ -16986,10 +17024,10 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B67" s="2" t="s">
         <v>151</v>
-      </c>
-      <c r="B67" s="2" t="s">
-        <v>152</v>
       </c>
       <c r="C67" s="2" t="s">
         <v>70</v>
@@ -16998,15 +17036,15 @@
         <v>74</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B68" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="B68" s="2" t="s">
-        <v>155</v>
       </c>
       <c r="C68" s="2" t="s">
         <v>70</v>
@@ -17015,15 +17053,15 @@
         <v>74</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B69" s="2" t="s">
         <v>156</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>157</v>
       </c>
       <c r="C69" s="2" t="s">
         <v>70</v>
@@ -17032,15 +17070,15 @@
         <v>74</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B70" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="B70" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="C70" s="2" t="s">
         <v>70</v>
@@ -17049,15 +17087,15 @@
         <v>74</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="B71" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="B71" s="2" t="s">
-        <v>161</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>70</v>
@@ -17066,58 +17104,58 @@
         <v>74</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B72" s="2" t="s">
         <v>162</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>163</v>
       </c>
       <c r="C72" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="C73" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D73" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C74" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.35">
@@ -17125,47 +17163,47 @@
         <v>172</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C75" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D75" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>167</v>
+        <v>444</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C76" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C77" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D77" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>167</v>
@@ -17173,16 +17211,16 @@
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C78" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>167</v>
@@ -17190,16 +17228,16 @@
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C79" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>167</v>
@@ -17207,16 +17245,16 @@
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C80" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>167</v>
@@ -17224,118 +17262,118 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C81" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C82" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C83" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C84" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C85" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
-        <v>195</v>
+        <v>164</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>196</v>
+        <v>165</v>
       </c>
       <c r="C87" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>167</v>
@@ -17343,16 +17381,16 @@
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B88" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>198</v>
       </c>
       <c r="C88" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D88" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>167</v>
@@ -17360,16 +17398,16 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B89" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>200</v>
       </c>
       <c r="C89" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D89" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>167</v>
@@ -17377,16 +17415,16 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B90" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>202</v>
       </c>
       <c r="C90" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D90" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>167</v>
@@ -17394,16 +17432,16 @@
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B91" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>204</v>
       </c>
       <c r="C91" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D91" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>167</v>
@@ -17411,2042 +17449,2042 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B92" s="2" t="s">
         <v>205</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>206</v>
       </c>
       <c r="C92" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D92" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B93" s="2" t="s">
         <v>208</v>
-      </c>
-      <c r="B93" s="2" t="s">
-        <v>209</v>
       </c>
       <c r="C93" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="B94" s="2" t="s">
         <v>210</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>211</v>
       </c>
       <c r="C94" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B95" s="2" t="s">
         <v>212</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>213</v>
       </c>
       <c r="C95" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D95" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="E95" s="2" t="s">
         <v>214</v>
-      </c>
-      <c r="E95" s="2" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="B96" s="2" t="s">
         <v>216</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>217</v>
       </c>
       <c r="C96" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B97" s="2" t="s">
         <v>219</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>220</v>
       </c>
       <c r="C97" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C98" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="B99" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="B99" s="2" t="s">
-        <v>223</v>
       </c>
       <c r="C99" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B100" s="2" t="s">
         <v>225</v>
-      </c>
-      <c r="B100" s="2" t="s">
-        <v>226</v>
       </c>
       <c r="C100" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D100" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E100" s="2" t="s">
         <v>227</v>
-      </c>
-      <c r="E100" s="2" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C101" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="B102" s="2" t="s">
         <v>230</v>
-      </c>
-      <c r="B102" s="2" t="s">
-        <v>231</v>
       </c>
       <c r="C102" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="B103" s="2" t="s">
         <v>233</v>
-      </c>
-      <c r="B103" s="2" t="s">
-        <v>234</v>
       </c>
       <c r="C103" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="B104" s="2" t="s">
         <v>236</v>
-      </c>
-      <c r="B104" s="2" t="s">
-        <v>237</v>
       </c>
       <c r="C104" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D104" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E104" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="E104" s="2" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
+        <v>239</v>
+      </c>
+      <c r="B105" s="2" t="s">
         <v>240</v>
-      </c>
-      <c r="B105" s="2" t="s">
-        <v>241</v>
       </c>
       <c r="C105" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D105" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E105" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="E105" s="2" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="B106" s="2" t="s">
         <v>242</v>
-      </c>
-      <c r="B106" s="2" t="s">
-        <v>243</v>
       </c>
       <c r="C106" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D106" s="2" t="s">
+        <v>237</v>
+      </c>
+      <c r="E106" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="E106" s="2" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B107" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="B107" s="2" t="s">
-        <v>245</v>
       </c>
       <c r="C107" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B108" s="2" t="s">
         <v>247</v>
-      </c>
-      <c r="B108" s="2" t="s">
-        <v>248</v>
       </c>
       <c r="C108" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C109" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="B110" s="2" t="s">
         <v>250</v>
-      </c>
-      <c r="B110" s="2" t="s">
-        <v>251</v>
       </c>
       <c r="C110" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B111" s="2" t="s">
         <v>253</v>
-      </c>
-      <c r="B111" s="2" t="s">
-        <v>254</v>
       </c>
       <c r="C111" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B112" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="B112" s="2" t="s">
-        <v>256</v>
       </c>
       <c r="C112" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="113" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B113" s="2" t="s">
         <v>257</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>258</v>
       </c>
       <c r="C113" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D113" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E113" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="114" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C114" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D114" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E114" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="115" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C115" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D115" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E115" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="116" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C116" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D116" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E116" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="117" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
+        <v>263</v>
+      </c>
+      <c r="B117" s="2" t="s">
         <v>264</v>
-      </c>
-      <c r="B117" s="2" t="s">
-        <v>265</v>
       </c>
       <c r="C117" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="118" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="B118" s="2" t="s">
         <v>266</v>
-      </c>
-      <c r="B118" s="2" t="s">
-        <v>267</v>
       </c>
       <c r="C118" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="119" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B119" s="2" t="s">
         <v>268</v>
-      </c>
-      <c r="B119" s="2" t="s">
-        <v>269</v>
       </c>
       <c r="C119" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="B120" s="2" t="s">
         <v>270</v>
-      </c>
-      <c r="B120" s="2" t="s">
-        <v>271</v>
       </c>
       <c r="C120" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="121" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="B121" s="2" t="s">
         <v>272</v>
-      </c>
-      <c r="B121" s="2" t="s">
-        <v>273</v>
       </c>
       <c r="C121" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="122" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C122" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D122" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="E122" s="2" t="s">
         <v>259</v>
-      </c>
-      <c r="E122" s="2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="123" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C123" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
+        <v>275</v>
+      </c>
+      <c r="B124" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="125" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
+        <v>278</v>
+      </c>
+      <c r="B125" s="2" t="s">
         <v>279</v>
-      </c>
-      <c r="B125" s="2" t="s">
-        <v>280</v>
       </c>
       <c r="C125" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="126" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="B126" s="2" t="s">
         <v>281</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>282</v>
       </c>
       <c r="C126" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
+        <v>282</v>
+      </c>
+      <c r="B127" s="2" t="s">
         <v>283</v>
-      </c>
-      <c r="B127" s="2" t="s">
-        <v>284</v>
       </c>
       <c r="C127" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="128" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
+        <v>284</v>
+      </c>
+      <c r="B128" s="2" t="s">
         <v>285</v>
-      </c>
-      <c r="B128" s="2" t="s">
-        <v>286</v>
       </c>
       <c r="C128" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
+        <v>286</v>
+      </c>
+      <c r="B129" s="2" t="s">
         <v>287</v>
-      </c>
-      <c r="B129" s="2" t="s">
-        <v>288</v>
       </c>
       <c r="C129" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B130" s="2" t="s">
         <v>289</v>
-      </c>
-      <c r="B130" s="2" t="s">
-        <v>290</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B131" s="2" t="s">
         <v>291</v>
-      </c>
-      <c r="B131" s="2" t="s">
-        <v>292</v>
       </c>
       <c r="C131" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B132" s="2" t="s">
         <v>293</v>
-      </c>
-      <c r="B132" s="2" t="s">
-        <v>294</v>
       </c>
       <c r="C132" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
+        <v>294</v>
+      </c>
+      <c r="B133" s="2" t="s">
         <v>295</v>
-      </c>
-      <c r="B133" s="2" t="s">
-        <v>296</v>
       </c>
       <c r="C133" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C134" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C135" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
+        <v>301</v>
+      </c>
+      <c r="B136" s="2" t="s">
         <v>302</v>
-      </c>
-      <c r="B136" s="2" t="s">
-        <v>303</v>
       </c>
       <c r="C136" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E136" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B137" s="2" t="s">
         <v>304</v>
-      </c>
-      <c r="B137" s="2" t="s">
-        <v>305</v>
       </c>
       <c r="C137" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B138" s="2" t="s">
         <v>306</v>
-      </c>
-      <c r="B138" s="2" t="s">
-        <v>307</v>
       </c>
       <c r="C138" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D138" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E138" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B139" s="2" t="s">
         <v>308</v>
-      </c>
-      <c r="B139" s="2" t="s">
-        <v>309</v>
       </c>
       <c r="C139" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D139" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B140" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="B140" s="2" t="s">
-        <v>311</v>
       </c>
       <c r="C140" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D140" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B141" s="2" t="s">
         <v>315</v>
-      </c>
-      <c r="B141" s="2" t="s">
-        <v>316</v>
       </c>
       <c r="C141" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D141" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A142" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B142" s="2" t="s">
         <v>317</v>
-      </c>
-      <c r="B142" s="2" t="s">
-        <v>318</v>
       </c>
       <c r="C142" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D142" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="B143" s="2" t="s">
         <v>319</v>
-      </c>
-      <c r="B143" s="2" t="s">
-        <v>320</v>
       </c>
       <c r="C143" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D143" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="B144" s="2" t="s">
         <v>321</v>
-      </c>
-      <c r="B144" s="2" t="s">
-        <v>322</v>
       </c>
       <c r="C144" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D144" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E144" s="2" t="s">
         <v>312</v>
-      </c>
-      <c r="E144" s="2" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D145" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E145" s="2" t="s">
         <v>312</v>
-      </c>
-      <c r="E145" s="2" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C146" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D146" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E146" s="2" t="s">
         <v>312</v>
-      </c>
-      <c r="E146" s="2" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="B147" s="2" t="s">
         <v>325</v>
-      </c>
-      <c r="B147" s="2" t="s">
-        <v>326</v>
       </c>
       <c r="C147" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="2" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C148" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D148" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="B149" s="2" t="s">
         <v>328</v>
-      </c>
-      <c r="B149" s="2" t="s">
-        <v>329</v>
       </c>
       <c r="C149" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D149" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B150" s="2" t="s">
         <v>330</v>
-      </c>
-      <c r="B150" s="2" t="s">
-        <v>331</v>
       </c>
       <c r="C150" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D150" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E150" s="2" t="s">
         <v>312</v>
-      </c>
-      <c r="E150" s="2" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B151" s="2" t="s">
         <v>332</v>
-      </c>
-      <c r="B151" s="2" t="s">
-        <v>333</v>
       </c>
       <c r="C151" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D151" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E151" s="2" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="B152" s="2" t="s">
         <v>334</v>
-      </c>
-      <c r="B152" s="2" t="s">
-        <v>335</v>
       </c>
       <c r="C152" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D152" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="E152" s="2" t="s">
         <v>312</v>
-      </c>
-      <c r="E152" s="2" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="B153" s="2" t="s">
         <v>336</v>
-      </c>
-      <c r="B153" s="2" t="s">
-        <v>337</v>
       </c>
       <c r="C153" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D153" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C154" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D154" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="E154" s="2" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="B155" s="2" t="s">
         <v>339</v>
-      </c>
-      <c r="B155" s="2" t="s">
-        <v>340</v>
       </c>
       <c r="C155" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D155" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="B156" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="B156" s="2" t="s">
-        <v>342</v>
-      </c>
       <c r="C156" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D156" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="E156" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="B157" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="B157" s="2" t="s">
-        <v>344</v>
-      </c>
       <c r="C157" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D157" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="B158" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="B158" s="3" t="s">
-        <v>346</v>
-      </c>
       <c r="C158" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E158" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="B159" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="B159" s="2" t="s">
-        <v>348</v>
-      </c>
       <c r="C159" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E159" s="2" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="B160" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="B160" s="2" t="s">
-        <v>350</v>
-      </c>
       <c r="C160" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E160" s="3" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="B161" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="B161" s="2" t="s">
-        <v>352</v>
-      </c>
       <c r="C161" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="E162" s="2" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="B163" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="B163" s="2" t="s">
+      <c r="C163" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D163" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="C163" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="D163" s="3" t="s">
-        <v>356</v>
-      </c>
       <c r="E163" s="2" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B164" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="B164" s="2" t="s">
-        <v>358</v>
-      </c>
       <c r="C164" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E164" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B165" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="B165" s="2" t="s">
-        <v>360</v>
-      </c>
       <c r="C165" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E165" s="2" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B166" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="B166" s="2" t="s">
-        <v>362</v>
-      </c>
       <c r="C166" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E166" s="2" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="B167" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="B167" s="2" t="s">
-        <v>364</v>
-      </c>
       <c r="C167" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E167" s="3" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B168" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="B168" s="2" t="s">
-        <v>366</v>
-      </c>
       <c r="C168" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E168" s="3" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="B169" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="B169" s="2" t="s">
-        <v>368</v>
-      </c>
       <c r="C169" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E169" s="2" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B170" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="B170" s="2" t="s">
-        <v>370</v>
-      </c>
       <c r="C170" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E170" s="2" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="B171" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="B171" s="2" t="s">
-        <v>372</v>
-      </c>
       <c r="C171" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="B172" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="B172" s="2" t="s">
-        <v>374</v>
-      </c>
       <c r="C172" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E172" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="E173" s="3" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B174" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="B174" s="2" t="s">
+      <c r="C174" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="D174" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="C174" s="2" t="s">
-        <v>342</v>
-      </c>
-      <c r="D174" s="2" t="s">
-        <v>378</v>
-      </c>
       <c r="E174" s="2" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="B175" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="B175" s="2" t="s">
-        <v>380</v>
-      </c>
       <c r="C175" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D175" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D176" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="E176" s="2" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="B177" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="B177" s="2" t="s">
+      <c r="C177" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="C177" s="2" t="s">
-        <v>384</v>
-      </c>
       <c r="D177" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="E177" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="B178" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C178" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="D178" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="B178" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="C178" s="2" t="s">
-        <v>384</v>
-      </c>
-      <c r="D178" s="2" t="s">
-        <v>386</v>
-      </c>
       <c r="E178" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D179" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E179" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="180" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D180" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E180" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="181" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D181" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="E181" s="2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="182" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="B182" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="B182" s="2" t="s">
-        <v>391</v>
-      </c>
       <c r="C182" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D182" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E182" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="183" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D183" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="E183" s="2" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B184" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="B184" s="2" t="s">
-        <v>394</v>
-      </c>
       <c r="C184" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E184" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="185" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="B185" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C185" s="2" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="D185" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="B186" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="B186" s="2" t="s">
+      <c r="C186" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="C186" s="2" t="s">
-        <v>398</v>
-      </c>
       <c r="D186" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="E186" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="187" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="B187" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="B187" s="2" t="s">
+      <c r="C187" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D187" s="3" t="s">
         <v>400</v>
       </c>
-      <c r="C187" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="D187" s="3" t="s">
-        <v>401</v>
-      </c>
       <c r="E187" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="188" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D188" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E188" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="189" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D189" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="E189" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="B190" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="B190" s="2" t="s">
+      <c r="C190" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D190" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="C190" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="D190" s="2" t="s">
-        <v>406</v>
-      </c>
       <c r="E190" s="2" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="191" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="B191" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="C191" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D191" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E191" s="2" t="s">
         <v>407</v>
-      </c>
-      <c r="B191" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="C191" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="D191" s="2" t="s">
-        <v>406</v>
-      </c>
-      <c r="E191" s="2" t="s">
-        <v>408</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
       <c r="B192" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C192" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D192" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E192" s="2" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
       <c r="B193" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="C193" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D193" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E193" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="194" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="B194" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C194" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D194" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E194" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="195" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="B195" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="B195" s="2" t="s">
-        <v>413</v>
-      </c>
       <c r="C195" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D195" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E195" s="2" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="196" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="B196" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="B196" s="2" t="s">
-        <v>415</v>
-      </c>
       <c r="C196" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D196" s="2" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="E196" s="2" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="197" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="B197" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="B197" s="2" t="s">
-        <v>417</v>
-      </c>
       <c r="C197" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D197" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E197" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A198" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="B198" s="3" t="s">
         <v>418</v>
       </c>
-      <c r="B198" s="3" t="s">
-        <v>419</v>
-      </c>
       <c r="C198" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E198" s="3" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="B199" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="B199" s="2" t="s">
-        <v>421</v>
-      </c>
       <c r="C199" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E199" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
       <c r="B200" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C200" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D200" s="2" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
       <c r="E200" s="2" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="201" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="B201" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="B201" s="2" t="s">
+      <c r="C201" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="D201" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="C201" s="2" t="s">
-        <v>398</v>
-      </c>
-      <c r="D201" s="2" t="s">
-        <v>425</v>
-      </c>
       <c r="E201" s="2" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="202" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="B202" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="C202" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D202" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E202" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B203" s="2" t="s">
         <v>427</v>
       </c>
-      <c r="B203" s="2" t="s">
-        <v>428</v>
-      </c>
       <c r="C203" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D203" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E203" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="204" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
       <c r="B204" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C204" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D204" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E204" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A205" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="B205" s="2" t="s">
         <v>431</v>
       </c>
-      <c r="B205" s="2" t="s">
-        <v>432</v>
-      </c>
       <c r="C205" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D205" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E205" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="B206" s="2" t="s">
         <v>433</v>
       </c>
-      <c r="B206" s="2" t="s">
-        <v>434</v>
-      </c>
       <c r="C206" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D206" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E206" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="B207" s="2" t="s">
         <v>435</v>
       </c>
-      <c r="B207" s="2" t="s">
-        <v>436</v>
-      </c>
       <c r="C207" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D207" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E207" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="B208" s="2" t="s">
         <v>437</v>
       </c>
-      <c r="B208" s="2" t="s">
-        <v>438</v>
-      </c>
       <c r="C208" s="2" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D208" s="2" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
       <c r="E208" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="B209" s="2" t="s">
         <v>439</v>
       </c>
-      <c r="B209" s="2" t="s">
-        <v>440</v>
-      </c>
       <c r="C209" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="D209" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="E209" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="B210" s="2" t="s">
         <v>441</v>
       </c>
-      <c r="B210" s="2" t="s">
-        <v>442</v>
-      </c>
       <c r="C210" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="D210" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E210" s="2" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="B211" s="2" t="s">
         <v>443</v>
       </c>
-      <c r="B211" s="2" t="s">
-        <v>444</v>
-      </c>
       <c r="C211" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="D211" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="E211" s="3" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.35">
@@ -19496,10 +19534,13 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F211" xr:uid="{6E49FC2C-E50A-494E-B408-F767D9411FB5}"/>
+  <conditionalFormatting sqref="A227:A1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A203">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A227:A1048576 A204:A211 A1:A202">
+  <conditionalFormatting sqref="A204:A211 A1:A202">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>